<commit_message>
docs(cost): CloudFront price by user region and initial volume estimate
- Workbook: choose the users' region (North America or South America)
  for CloudFront data transfer and HTTPS request prices (AWS Price List
  API); API Gateway stays on us-east-1 prices. Example rows replaced by
  the initial one-day estimate (200k images, 10k APKs).
- ADR: cost reading kept short: small on-demand gap, region can flip it
  (South America edges cost more than us-east-1 egress), flat-rate CDN
  plan is cheaper but blocked by the governance requirement.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/custo/apigw-vs-cloudfront.xlsx
+++ b/docs/custo/apigw-vs-cloudfront.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\apigw-transfer\.claude\worktrees\project-proposal-code-review-f9ab5f\docs\custo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8349F550-6D0B-4418-9FE6-952240638D1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0311FFE3-C7F4-44D2-AE7D-AFC432F1516C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -219,7 +219,35 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>https://aws.amazon.com/cloudfront/pricing/ (América do Norte/Europa)</t>
+          <t>CloudFront cobra pela região do edge que atende o usuário. API Gateway cobra pela região da API (us-east-1).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000E000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>https://aws.amazon.com/cloudfront/pricing/ (AWS Price List API)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-00000F000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color theme="1"/>
+            <rFont val="Calibri"/>
+            <family val="2"/>
+            <scheme val="minor"/>
+          </rPr>
+          <t>https://aws.amazon.com/cloudfront/pricing/ (AWS Price List API)</t>
         </r>
       </text>
     </comment>
@@ -252,7 +280,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="130">
   <si>
     <t>Consumo medido em produção</t>
   </si>
@@ -260,7 +288,7 @@
     <t>Dias cobertos pelo levantamento</t>
   </si>
   <si>
-    <t>Preencha as colunas amarelas (C a F). As linhas 5 e 6 são exemplos: substitua pelos dados reais.</t>
+    <t>Preencha as colunas amarelas (C a F). Linhas 5 e 6: estimativa inicial de 1 dia, substituir pelo levantamento.</t>
   </si>
   <si>
     <t>Categoria de arquivo</t>
@@ -290,10 +318,10 @@
     <t>Requisições CloudFront no período</t>
   </si>
   <si>
-    <t>Imagens (exemplo)</t>
-  </si>
-  <si>
-    <t>APKs (exemplo)</t>
+    <t>Imagens (estimativa)</t>
+  </si>
+  <si>
+    <t>APKs (estimativa)</t>
   </si>
   <si>
     <t>Total no período</t>
@@ -314,10 +342,10 @@
     <t>Como usar</t>
   </si>
   <si>
-    <t>1. Aba Consumo: informe quantos dias o levantamento cobre (célula C2) e, por categoria de arquivo, downloads no período, tamanho médio, % com HEAD e % de requisições extras (retomadas/retries). Células amarelas com texto azul são entradas. As duas linhas preenchidas são exemplos: substitua pelos dados reais.</t>
-  </si>
-  <si>
-    <t>2. Aba Premissas: preços e parâmetros (texto azul). Ajuste se a região ou os preços forem outros (ex.: bucket/API em sa-east-1, usuários na América do Sul).</t>
+    <t>1. Aba Consumo: informe quantos dias o levantamento cobre (célula C2) e, por categoria de arquivo, downloads no período, tamanho médio, % com HEAD e % de requisições extras (retomadas/retries). Células amarelas com texto azul são entradas. As duas linhas preenchidas são uma estimativa inicial: substitua pelo levantamento.</t>
+  </si>
+  <si>
+    <t>2. Aba Premissas: escolha a região dos usuários (América do Norte ou América do Sul), que define o preço do CloudFront. O API Gateway usa o preço de us-east-1. Demais preços e parâmetros são editáveis (texto azul).</t>
   </si>
   <si>
     <t>3. Aba Comparativo: resultado mensal, sem nada a preencher.</t>
@@ -365,7 +393,7 @@
     <t>Lambda: https://aws.amazon.com/lambda/pricing/</t>
   </si>
   <si>
-    <t>Preço de referência us-east-1 / América do Norte, conferido em 2026-09-13. Confirmar na página antes de decidir.</t>
+    <t>Preços de referência (API Gateway/S3/Lambda em us-east-1; CloudFront por região), conferidos em 2026-09-13. Confirmar antes de decidir.</t>
   </si>
   <si>
     <t>Premissas e preços</t>
@@ -419,7 +447,16 @@
     <t>Free tier de requisições (por mês)</t>
   </si>
   <si>
-    <t>Preço por 10.000 requisições HTTPS ($)</t>
+    <t>Região dos usuários (define a tabela de preço do CloudFront)</t>
+  </si>
+  <si>
+    <t>América do Norte</t>
+  </si>
+  <si>
+    <t>Preço por 10.000 requisições HTTPS ($) - América do Norte</t>
+  </si>
+  <si>
+    <t>Preço por 10.000 requisições HTTPS ($) - América do Sul</t>
   </si>
   <si>
     <t>API Gateway REST: requisições por mês (preço por milhão)</t>
@@ -476,7 +513,7 @@
     <t>Fonte: https://aws.amazon.com/api-gateway/pricing/ (mesma tabela de transferência do EC2, us-east-1). Última faixa com 'Até' = 1E+12 (sem limite).</t>
   </si>
   <si>
-    <t>CloudFront sob demanda: transferência para a internet por mês (preço por GB, após free tier)</t>
+    <t>CloudFront sob demanda - América do Norte: transferência por mês (preço por GB, após free tier)</t>
   </si>
   <si>
     <t>Próximos 350 TB</t>
@@ -488,7 +525,13 @@
     <t>Acima de 1 PB</t>
   </si>
   <si>
-    <t>Fonte: https://aws.amazon.com/cloudfront/pricing/ (América do Norte; América do Sul é mais cara, confirmar). Última faixa com 'Até' = 1E+12 (sem limite).</t>
+    <t>Fonte: https://aws.amazon.com/cloudfront/pricing/ (AWS Price List API, United States). Última faixa com 'Até' = 1E+12 (sem limite).</t>
+  </si>
+  <si>
+    <t>CloudFront sob demanda - América do Sul: transferência por mês (preço por GB, após free tier)</t>
+  </si>
+  <si>
+    <t>Fonte: https://aws.amazon.com/cloudfront/pricing/ (AWS Price List API, South America). Última faixa com 'Até' = 1E+12 (sem limite).</t>
   </si>
   <si>
     <t>CloudFront planos de preço fixo (sem cobrança excedente)</t>
@@ -576,6 +619,9 @@
   </si>
   <si>
     <t>Requisições (acima do free tier)</t>
+  </si>
+  <si>
+    <t>Preço conforme a região dos usuários (Premissas)</t>
   </si>
   <si>
     <t>Transferência para a internet (acima do free tier)</t>
@@ -746,7 +792,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -766,6 +812,7 @@
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1239,7 +1286,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1440,454 +1487,609 @@
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="12">
-        <v>0.01</v>
+      <c r="C20" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
+      <c r="B21" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="12">
+        <v>0.01</v>
+      </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="B22" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
+      <c r="B22" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="12">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="B23" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="D23" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>60</v>
-      </c>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C24" s="9">
-        <v>0</v>
-      </c>
-      <c r="D24" s="9">
-        <v>333</v>
-      </c>
-      <c r="E24" s="12">
-        <v>3.5</v>
-      </c>
+      <c r="B24" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C25" s="9">
-        <v>333</v>
-      </c>
-      <c r="D25" s="9">
-        <v>1000</v>
-      </c>
-      <c r="E25" s="12">
-        <v>2.8</v>
+      <c r="E25" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="4"/>
-      <c r="B26" s="14" t="s">
-        <v>63</v>
+      <c r="B26" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="C26" s="9">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D26" s="9">
-        <v>20000</v>
+        <v>333</v>
       </c>
       <c r="E26" s="12">
-        <v>2.38</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
-      <c r="B27" s="14" t="s">
-        <v>64</v>
+      <c r="B27" s="15" t="s">
+        <v>65</v>
       </c>
       <c r="C27" s="9">
-        <v>20000</v>
+        <v>333</v>
       </c>
       <c r="D27" s="9">
-        <v>1000000000000</v>
+        <v>1000</v>
       </c>
       <c r="E27" s="12">
-        <v>1.51</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
-      <c r="B28" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
+      <c r="B28" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="9">
+        <v>1000</v>
+      </c>
+      <c r="D28" s="9">
+        <v>20000</v>
+      </c>
+      <c r="E28" s="12">
+        <v>2.38</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
-      <c r="B29" s="4"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
+      <c r="B29" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="9">
+        <v>20000</v>
+      </c>
+      <c r="D29" s="9">
+        <v>1000000000000</v>
+      </c>
+      <c r="E29" s="12">
+        <v>1.51</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
-      <c r="B30" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
+      <c r="B30" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
-      <c r="B31" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C31" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D31" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>60</v>
-      </c>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="9">
-        <v>0</v>
-      </c>
-      <c r="D32" s="9">
-        <v>10240</v>
-      </c>
-      <c r="E32" s="12">
-        <v>0.09</v>
-      </c>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C33" s="9">
-        <v>10240</v>
-      </c>
-      <c r="D33" s="9">
-        <v>51200</v>
-      </c>
-      <c r="E33" s="12">
-        <v>8.5000000000000006E-2</v>
+      <c r="D33" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
-      <c r="B34" s="14" t="s">
-        <v>71</v>
+      <c r="B34" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="C34" s="9">
-        <v>51200</v>
+        <v>0</v>
       </c>
       <c r="D34" s="9">
-        <v>153600</v>
+        <v>10240</v>
       </c>
       <c r="E34" s="12">
-        <v>7.0000000000000007E-2</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="14" t="s">
-        <v>72</v>
+      <c r="B35" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C35" s="9">
-        <v>153600</v>
+        <v>10240</v>
       </c>
       <c r="D35" s="9">
-        <v>1000000000000</v>
+        <v>51200</v>
       </c>
       <c r="E35" s="12">
-        <v>0.05</v>
+        <v>8.5000000000000006E-2</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4"/>
-      <c r="E36" s="4"/>
+      <c r="B36" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C36" s="9">
+        <v>51200</v>
+      </c>
+      <c r="D36" s="9">
+        <v>153600</v>
+      </c>
+      <c r="E36" s="12">
+        <v>7.0000000000000007E-2</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
+      <c r="B37" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="C37" s="9">
+        <v>153600</v>
+      </c>
+      <c r="D37" s="9">
+        <v>1000000000000</v>
+      </c>
+      <c r="E37" s="12">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
-      <c r="B38" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
+      <c r="B38" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
-      <c r="B39" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="C39" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D39" s="13" t="s">
-        <v>68</v>
-      </c>
-      <c r="E39" s="13" t="s">
-        <v>60</v>
-      </c>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
-      <c r="B40" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C40" s="9">
-        <v>0</v>
-      </c>
-      <c r="D40" s="9">
-        <v>10240</v>
-      </c>
-      <c r="E40" s="12">
-        <v>8.5000000000000006E-2</v>
-      </c>
+      <c r="B40" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C41" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C41" s="9">
-        <v>10240</v>
-      </c>
-      <c r="D41" s="9">
-        <v>51200</v>
-      </c>
-      <c r="E41" s="12">
-        <v>0.08</v>
+      <c r="D41" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E41" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
-      <c r="B42" s="14" t="s">
-        <v>71</v>
+      <c r="B42" s="15" t="s">
+        <v>72</v>
       </c>
       <c r="C42" s="9">
-        <v>51200</v>
+        <v>0</v>
       </c>
       <c r="D42" s="9">
-        <v>153600</v>
+        <v>10240</v>
       </c>
       <c r="E42" s="12">
-        <v>0.06</v>
+        <v>8.5000000000000006E-2</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" s="4"/>
-      <c r="B43" s="14" t="s">
-        <v>75</v>
+      <c r="B43" s="15" t="s">
+        <v>73</v>
       </c>
       <c r="C43" s="9">
-        <v>153600</v>
+        <v>10240</v>
       </c>
       <c r="D43" s="9">
-        <v>512000</v>
+        <v>51200</v>
       </c>
       <c r="E43" s="12">
-        <v>0.04</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
-      <c r="B44" s="14" t="s">
-        <v>76</v>
+      <c r="B44" s="15" t="s">
+        <v>74</v>
       </c>
       <c r="C44" s="9">
-        <v>512000</v>
+        <v>51200</v>
       </c>
       <c r="D44" s="9">
-        <v>1048576</v>
+        <v>153600</v>
       </c>
       <c r="E44" s="12">
-        <v>0.03</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
-      <c r="B45" s="14" t="s">
-        <v>77</v>
+      <c r="B45" s="15" t="s">
+        <v>78</v>
       </c>
       <c r="C45" s="9">
-        <v>1048576</v>
+        <v>153600</v>
       </c>
       <c r="D45" s="9">
-        <v>1000000000000</v>
+        <v>512000</v>
       </c>
       <c r="E45" s="12">
-        <v>2.5000000000000001E-2</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
-      <c r="B46" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
+      <c r="B46" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="9">
+        <v>512000</v>
+      </c>
+      <c r="D46" s="9">
+        <v>1048576</v>
+      </c>
+      <c r="E46" s="12">
+        <v>0.03</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
-      <c r="B47" s="4"/>
-      <c r="C47" s="4"/>
-      <c r="D47" s="4"/>
-      <c r="E47" s="4"/>
+      <c r="B47" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C47" s="9">
+        <v>1048576</v>
+      </c>
+      <c r="D47" s="9">
+        <v>1000000000000</v>
+      </c>
+      <c r="E47" s="12">
+        <v>2.5000000000000001E-2</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
-      <c r="B48" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-    </row>
-    <row r="49" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="B48" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="4"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
-      <c r="B49" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="C49" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D49" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="E49" s="13" t="s">
-        <v>83</v>
-      </c>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="4"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
-      <c r="B50" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C50" s="11">
-        <v>0</v>
-      </c>
-      <c r="D50" s="9">
-        <v>1000000</v>
-      </c>
-      <c r="E50" s="9">
-        <v>100</v>
-      </c>
+      <c r="B50" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
-      <c r="B51" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C51" s="11">
-        <v>15</v>
-      </c>
-      <c r="D51" s="9">
-        <v>10000000</v>
-      </c>
-      <c r="E51" s="9">
-        <v>51200</v>
+      <c r="B51" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D51" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
       <c r="B52" s="15" t="s">
-        <v>86</v>
-      </c>
-      <c r="C52" s="11">
-        <v>200</v>
+        <v>72</v>
+      </c>
+      <c r="C52" s="9">
+        <v>0</v>
       </c>
       <c r="D52" s="9">
-        <v>125000000</v>
-      </c>
-      <c r="E52" s="9">
-        <v>51200</v>
+        <v>10240</v>
+      </c>
+      <c r="E52" s="12">
+        <v>0.11</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="15" t="s">
+        <v>73</v>
+      </c>
+      <c r="C53" s="9">
+        <v>10240</v>
+      </c>
+      <c r="D53" s="9">
+        <v>51200</v>
+      </c>
+      <c r="E53" s="12">
+        <v>0.105</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="4"/>
+      <c r="B54" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C54" s="9">
+        <v>51200</v>
+      </c>
+      <c r="D54" s="9">
+        <v>153600</v>
+      </c>
+      <c r="E54" s="12">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="4"/>
+      <c r="B55" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="C55" s="9">
+        <v>153600</v>
+      </c>
+      <c r="D55" s="9">
+        <v>512000</v>
+      </c>
+      <c r="E55" s="12">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="4"/>
+      <c r="B56" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C56" s="9">
+        <v>512000</v>
+      </c>
+      <c r="D56" s="9">
+        <v>1048576</v>
+      </c>
+      <c r="E56" s="12">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="4"/>
+      <c r="B57" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C57" s="9">
+        <v>1048576</v>
+      </c>
+      <c r="D57" s="9">
+        <v>1000000000000</v>
+      </c>
+      <c r="E57" s="12">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="4"/>
+      <c r="B58" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C58" s="4"/>
+      <c r="D58" s="4"/>
+      <c r="E58" s="4"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+      <c r="D59" s="4"/>
+      <c r="E59" s="4"/>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="4"/>
+      <c r="B60" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="C60" s="8"/>
+      <c r="D60" s="8"/>
+      <c r="E60" s="8"/>
+    </row>
+    <row r="61" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="4"/>
+      <c r="B61" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C61" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D61" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="C53" s="11">
+      <c r="E61" s="14" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="4"/>
+      <c r="B62" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C62" s="11">
+        <v>0</v>
+      </c>
+      <c r="D62" s="9">
+        <v>1000000</v>
+      </c>
+      <c r="E62" s="9">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="16" t="s">
+        <v>90</v>
+      </c>
+      <c r="C63" s="11">
+        <v>15</v>
+      </c>
+      <c r="D63" s="9">
+        <v>10000000</v>
+      </c>
+      <c r="E63" s="9">
+        <v>51200</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="4"/>
+      <c r="B64" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="C64" s="11">
+        <v>200</v>
+      </c>
+      <c r="D64" s="9">
+        <v>125000000</v>
+      </c>
+      <c r="E64" s="9">
+        <v>51200</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="4"/>
+      <c r="B65" s="16" t="s">
+        <v>92</v>
+      </c>
+      <c r="C65" s="11">
         <v>1000</v>
       </c>
-      <c r="D53" s="9">
+      <c r="D65" s="9">
         <v>500000000</v>
       </c>
-      <c r="E53" s="9">
+      <c r="E65" s="9">
         <v>51200</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="4"/>
-      <c r="B54" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+    <row r="66" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="4"/>
+      <c r="B66" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="C66" s="4"/>
+      <c r="D66" s="4"/>
+      <c r="E66" s="4"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="decimal" error="Informe um valor entre 0 e 1 (ex.: 0,9 = 90%)." sqref="C9 C17" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations count="3">
+    <dataValidation type="list" error="Escolha América do Norte ou América do Sul." sqref="C20" xr:uid="{00000000-0002-0000-0100-000000000000}">
+      <formula1>"América do Norte,América do Sul"</formula1>
+    </dataValidation>
+    <dataValidation type="decimal" error="Informe um valor entre 0 e 1 (ex.: 0,9 = 90%)." sqref="C9 C17" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
-    <dataValidation type="whole" error="Use 1 (uma requisição por arquivo) ou 0 (mesmos blocos do API Gateway)." sqref="C7" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="whole" error="Use 1 (uma requisição por arquivo) ou 0 (mesmos blocos do API Gateway)." sqref="C7" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
@@ -1928,10 +2130,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="18">
+      <c r="C2" s="19">
         <v>1</v>
       </c>
       <c r="D2" s="6" t="s">
@@ -1958,438 +2160,438 @@
     </row>
     <row r="4" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="13" t="s">
+      <c r="D4" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="13" t="s">
+      <c r="F4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="G4" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="13" t="s">
+      <c r="H4" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="13" t="s">
+      <c r="J4" s="14" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
-      <c r="B5" s="19" t="s">
+      <c r="B5" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="18">
-        <v>50000</v>
-      </c>
-      <c r="D5" s="20">
+      <c r="C5" s="19">
+        <v>200000</v>
+      </c>
+      <c r="D5" s="21">
         <v>0.2</v>
       </c>
-      <c r="E5" s="21">
-        <v>0</v>
-      </c>
-      <c r="F5" s="21">
+      <c r="E5" s="22">
+        <v>0</v>
+      </c>
+      <c r="F5" s="22">
         <v>0.02</v>
       </c>
-      <c r="G5" s="22">
+      <c r="G5" s="23">
         <f t="shared" ref="G5:G19" si="0">C5*D5/1024</f>
-        <v>9.765625</v>
-      </c>
-      <c r="H5" s="23">
+        <v>39.0625</v>
+      </c>
+      <c r="H5" s="24">
         <f>IF(D5&gt;0,ROUNDUP(D5/Premissas!$C$6,0),0)</f>
         <v>1</v>
       </c>
-      <c r="I5" s="23">
+      <c r="I5" s="24">
         <f t="shared" ref="I5:I19" si="1">C5*(H5+E5)*(1+F5)</f>
-        <v>51000</v>
-      </c>
-      <c r="J5" s="23">
+        <v>204000</v>
+      </c>
+      <c r="J5" s="24">
         <f>C5*(IF(Premissas!$C$7=1,IF(D5&gt;0,1,0),H5)+E5)*(1+F5)</f>
-        <v>51000</v>
+        <v>204000</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="18">
-        <v>500</v>
-      </c>
-      <c r="D6" s="20">
+      <c r="C6" s="19">
+        <v>10000</v>
+      </c>
+      <c r="D6" s="21">
         <v>100</v>
       </c>
-      <c r="E6" s="21">
+      <c r="E6" s="22">
         <v>1</v>
       </c>
-      <c r="F6" s="21">
+      <c r="F6" s="22">
         <v>0.05</v>
       </c>
-      <c r="G6" s="22">
+      <c r="G6" s="23">
         <f t="shared" si="0"/>
-        <v>48.828125</v>
-      </c>
-      <c r="H6" s="23">
+        <v>976.5625</v>
+      </c>
+      <c r="H6" s="24">
         <f>IF(D6&gt;0,ROUNDUP(D6/Premissas!$C$6,0),0)</f>
         <v>13</v>
       </c>
-      <c r="I6" s="23">
+      <c r="I6" s="24">
         <f t="shared" si="1"/>
-        <v>7350</v>
-      </c>
-      <c r="J6" s="23">
+        <v>147000</v>
+      </c>
+      <c r="J6" s="24">
         <f>C6*(IF(Premissas!$C$7=1,IF(D6&gt;0,1,0),H6)+E6)*(1+F6)</f>
-        <v>1050</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="22">
+      <c r="B7" s="20"/>
+      <c r="C7" s="19"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H7" s="23">
+      <c r="H7" s="24">
         <f>IF(D7&gt;0,ROUNDUP(D7/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I7" s="23">
+      <c r="I7" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="24">
         <f>C7*(IF(Premissas!$C$7=1,IF(D7&gt;0,1,0),H7)+E7)*(1+F7)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21"/>
-      <c r="G8" s="22">
+      <c r="B8" s="20"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="21"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="22"/>
+      <c r="G8" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H8" s="23">
+      <c r="H8" s="24">
         <f>IF(D8&gt;0,ROUNDUP(D8/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I8" s="23">
+      <c r="I8" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J8" s="23">
+      <c r="J8" s="24">
         <f>C8*(IF(Premissas!$C$7=1,IF(D8&gt;0,1,0),H8)+E8)*(1+F8)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="4"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="22">
+      <c r="B9" s="20"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H9" s="23">
+      <c r="H9" s="24">
         <f>IF(D9&gt;0,ROUNDUP(D9/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="24">
         <f>C9*(IF(Premissas!$C$7=1,IF(D9&gt;0,1,0),H9)+E9)*(1+F9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="22">
+      <c r="B10" s="20"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H10" s="23">
+      <c r="H10" s="24">
         <f>IF(D10&gt;0,ROUNDUP(D10/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="23">
+      <c r="I10" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J10" s="23">
+      <c r="J10" s="24">
         <f>C10*(IF(Premissas!$C$7=1,IF(D10&gt;0,1,0),H10)+E10)*(1+F10)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="22">
+      <c r="B11" s="20"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H11" s="23">
+      <c r="H11" s="24">
         <f>IF(D11&gt;0,ROUNDUP(D11/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="23">
+      <c r="I11" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J11" s="23">
+      <c r="J11" s="24">
         <f>C11*(IF(Premissas!$C$7=1,IF(D11&gt;0,1,0),H11)+E11)*(1+F11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="18"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="22">
+      <c r="B12" s="20"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="23">
+      <c r="H12" s="24">
         <f>IF(D12&gt;0,ROUNDUP(D12/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I12" s="23">
+      <c r="I12" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J12" s="23">
+      <c r="J12" s="24">
         <f>C12*(IF(Premissas!$C$7=1,IF(D12&gt;0,1,0),H12)+E12)*(1+F12)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="22">
+      <c r="B13" s="20"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H13" s="23">
+      <c r="H13" s="24">
         <f>IF(D13&gt;0,ROUNDUP(D13/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I13" s="23">
+      <c r="I13" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J13" s="23">
+      <c r="J13" s="24">
         <f>C13*(IF(Premissas!$C$7=1,IF(D13&gt;0,1,0),H13)+E13)*(1+F13)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
-      <c r="B14" s="19"/>
-      <c r="C14" s="18"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="21"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="22">
+      <c r="B14" s="20"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="23">
+      <c r="H14" s="24">
         <f>IF(D14&gt;0,ROUNDUP(D14/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I14" s="23">
+      <c r="I14" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J14" s="23">
+      <c r="J14" s="24">
         <f>C14*(IF(Premissas!$C$7=1,IF(D14&gt;0,1,0),H14)+E14)*(1+F14)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="21"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="22">
+      <c r="B15" s="20"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H15" s="23">
+      <c r="H15" s="24">
         <f>IF(D15&gt;0,ROUNDUP(D15/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I15" s="23">
+      <c r="I15" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="24">
         <f>C15*(IF(Premissas!$C$7=1,IF(D15&gt;0,1,0),H15)+E15)*(1+F15)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="4"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="22">
+      <c r="B16" s="20"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="23">
+      <c r="H16" s="24">
         <f>IF(D16&gt;0,ROUNDUP(D16/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I16" s="23">
+      <c r="I16" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="24">
         <f>C16*(IF(Premissas!$C$7=1,IF(D16&gt;0,1,0),H16)+E16)*(1+F16)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="22">
+      <c r="B17" s="20"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H17" s="23">
+      <c r="H17" s="24">
         <f>IF(D17&gt;0,ROUNDUP(D17/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I17" s="23">
+      <c r="I17" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="24">
         <f>C17*(IF(Premissas!$C$7=1,IF(D17&gt;0,1,0),H17)+E17)*(1+F17)</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="21"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="22">
+      <c r="B18" s="20"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="23">
+      <c r="H18" s="24">
         <f>IF(D18&gt;0,ROUNDUP(D18/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I18" s="23">
+      <c r="I18" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J18" s="23">
+      <c r="J18" s="24">
         <f>C18*(IF(Premissas!$C$7=1,IF(D18&gt;0,1,0),H18)+E18)*(1+F18)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="22">
+      <c r="B19" s="20"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="23">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H19" s="23">
+      <c r="H19" s="24">
         <f>IF(D19&gt;0,ROUNDUP(D19/Premissas!$C$6,0),0)</f>
         <v>0</v>
       </c>
-      <c r="I19" s="23">
+      <c r="I19" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="24">
         <f>C19*(IF(Premissas!$C$7=1,IF(D19&gt;0,1,0),H19)+E19)*(1+F19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="24">
+      <c r="C20" s="25">
         <f>SUM(C5:C19)</f>
-        <v>50500</v>
+        <v>210000</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
-      <c r="G20" s="25">
+      <c r="G20" s="26">
         <f>SUM(G5:G19)</f>
-        <v>58.59375</v>
+        <v>1015.625</v>
       </c>
       <c r="H20" s="4"/>
-      <c r="I20" s="24">
+      <c r="I20" s="25">
         <f>SUM(I5:I19)</f>
-        <v>58350</v>
-      </c>
-      <c r="J20" s="24">
+        <v>351000</v>
+      </c>
+      <c r="J20" s="25">
         <f>SUM(J5:J19)</f>
-        <v>52050</v>
+        <v>225000</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -2406,29 +2608,29 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="4"/>
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35"/>
-      <c r="G22" s="35"/>
-      <c r="H22" s="35"/>
-      <c r="I22" s="35"/>
-      <c r="J22" s="35"/>
+      <c r="C22" s="36"/>
+      <c r="D22" s="36"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="36"/>
+      <c r="J22" s="36"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
-      <c r="B23" s="35"/>
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="35"/>
-      <c r="F23" s="35"/>
-      <c r="G23" s="35"/>
-      <c r="H23" s="35"/>
-      <c r="I23" s="35"/>
-      <c r="J23" s="35"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="36"/>
+      <c r="E23" s="36"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2462,7 +2664,7 @@
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
@@ -2470,7 +2672,7 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
       <c r="B2" s="6" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -2484,54 +2686,54 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="7" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
-      <c r="B5" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C5" s="26">
+      <c r="B5" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="27">
         <f>Consumo!$G$20*(Premissas!$C$5/Consumo!$C$2)</f>
-        <v>1757.8125</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>93</v>
+        <v>30468.75</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
-      <c r="B6" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" s="27">
+      <c r="B6" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="C6" s="28">
         <f>Consumo!$I$20*(Premissas!$C$5/Consumo!$C$2)</f>
-        <v>1750500</v>
+        <v>10530000</v>
       </c>
       <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
-      <c r="B7" s="14" t="s">
-        <v>95</v>
-      </c>
-      <c r="C7" s="27">
+      <c r="B7" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="28">
         <f>Consumo!$J$20*(Premissas!$C$5/Consumo!$C$2)</f>
-        <v>1561500</v>
+        <v>6750000</v>
       </c>
       <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
-      <c r="B8" s="14" t="s">
-        <v>96</v>
-      </c>
-      <c r="C8" s="27">
+      <c r="B8" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="28">
         <f>Consumo!$C$20*(Premissas!$C$5/Consumo!$C$2)</f>
-        <v>1515000</v>
+        <v>6300000</v>
       </c>
       <c r="D8" s="4"/>
     </row>
@@ -2544,69 +2746,69 @@
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="7" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
-      <c r="B11" s="14" t="s">
-        <v>98</v>
-      </c>
-      <c r="C11" s="28">
-        <f>SUMPRODUCT((($C$6/1000000)&gt;Premissas!$C$24:$C$27)*((($C$6/1000000)-Premissas!$C$24:$C$27)-(($C$6/1000000)&gt;Premissas!$D$24:$D$27)*(($C$6/1000000)-Premissas!$D$24:$D$27))*Premissas!$E$24:$E$27)</f>
-        <v>6.1267499999999995</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>99</v>
+      <c r="B11" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="C11" s="29">
+        <f>SUMPRODUCT((($C$6/1000000)&gt;Premissas!$C$26:$C$29)*((($C$6/1000000)-Premissas!$C$26:$C$29)-(($C$6/1000000)&gt;Premissas!$D$26:$D$29)*(($C$6/1000000)-Premissas!$D$26:$D$29))*Premissas!$E$26:$E$29)</f>
+        <v>36.854999999999997</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
-      <c r="B12" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C12" s="28">
-        <f>SUMPRODUCT(($C$5&gt;Premissas!$C$32:$C$35)*(($C$5-Premissas!$C$32:$C$35)-($C$5&gt;Premissas!$D$32:$D$35)*($C$5-Premissas!$D$32:$D$35))*Premissas!$E$32:$E$35)</f>
-        <v>158.203125</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>101</v>
+      <c r="B12" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="C12" s="29">
+        <f>SUMPRODUCT(($C$5&gt;Premissas!$C$34:$C$37)*(($C$5-Premissas!$C$34:$C$37)-($C$5&gt;Premissas!$D$34:$D$37)*($C$5-Premissas!$D$34:$D$37))*Premissas!$E$34:$E$37)</f>
+        <v>2641.0437499999998</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
-      <c r="B13" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="C13" s="28">
+      <c r="B13" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="29">
         <f>$C$6/1000*Premissas!$C$15</f>
-        <v>0.70020000000000004</v>
+        <v>4.2120000000000006</v>
       </c>
       <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
-      <c r="B14" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C14" s="28">
+      <c r="B14" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C14" s="29">
         <f>$C$6*(1-Premissas!$C$9)*(Premissas!$C$12/1000000+(Premissas!$C$10/1024)*(Premissas!$C$11/1000)*Premissas!$C$13)</f>
-        <v>0.10794764587499998</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>104</v>
+        <v>0.64935087749999987</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
-      <c r="B15" s="17" t="s">
-        <v>105</v>
-      </c>
-      <c r="C15" s="29">
+      <c r="B15" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="30">
         <f>SUM(C11:C14)</f>
-        <v>165.13802264587497</v>
+        <v>2682.7601008775</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -2619,54 +2821,56 @@
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
-      <c r="B18" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="C18" s="28">
-        <f>MAX(0,$C$7-Premissas!$C$19)/10000*Premissas!$C$20</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="4"/>
+      <c r="B18" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="29">
+        <f>MAX(0,$C$7-Premissas!$C$19)/10000*IF((Premissas!$C$20="América do Sul"),Premissas!$C$22,Premissas!$C$21)</f>
+        <v>0</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
-      <c r="B19" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="C19" s="28">
-        <f>SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$40:$C$45)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$40:$C$45)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$40:$D$45)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$40:$D$45))*Premissas!$E$40:$E$45)</f>
-        <v>62.374062500000008</v>
-      </c>
-      <c r="D19" s="16" t="s">
-        <v>109</v>
+      <c r="B19" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="29">
+        <f>IF((Premissas!$C$20="América do Sul"),SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$52:$C$57)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$52:$C$57)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$52:$D$57)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$52:$D$57))*Premissas!$E$52:$E$57),SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$42:$C$47)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$42:$C$47)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$42:$D$47)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$42:$D$47))*Premissas!$E$42:$E$47))</f>
+        <v>2406.7800000000002</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
-      <c r="B20" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="C20" s="28">
+      <c r="B20" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="C20" s="29">
         <f>$C$7*(1-Premissas!$C$17)/1000*Premissas!$C$15</f>
-        <v>0.12491999999999999</v>
+        <v>0.53999999999999992</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
-      <c r="B21" s="17" t="s">
-        <v>111</v>
-      </c>
-      <c r="C21" s="29">
+      <c r="B21" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="C21" s="30">
         <f>SUM(C18:C20)</f>
-        <v>62.498982500000011</v>
+        <v>2407.3200000000002</v>
       </c>
       <c r="D21" s="4"/>
     </row>
@@ -2679,31 +2883,31 @@
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="7" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
-      <c r="B24" s="14" t="s">
-        <v>113</v>
-      </c>
-      <c r="C24" s="30" t="str">
-        <f>IF(AND($C$7&lt;=Premissas!$D$50,$C$5&lt;=Premissas!$E$50),Premissas!$B$50,IF(AND($C$7&lt;=Premissas!$D$51,$C$5&lt;=Premissas!$E$51),Premissas!$B$51,IF(AND($C$7&lt;=Premissas!$D$52,$C$5&lt;=Premissas!$E$52),Premissas!$B$52,IF(AND($C$7&lt;=Premissas!$D$53,$C$5&lt;=Premissas!$E$53),Premissas!$B$53,"Excede os planos (usar sob demanda)"))))</f>
+      <c r="B24" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="C24" s="31" t="str">
+        <f>IF(AND($C$7&lt;=Premissas!$D$62,$C$5&lt;=Premissas!$E$62),Premissas!$B$62,IF(AND($C$7&lt;=Premissas!$D$63,$C$5&lt;=Premissas!$E$63),Premissas!$B$63,IF(AND($C$7&lt;=Premissas!$D$64,$C$5&lt;=Premissas!$E$64),Premissas!$B$64,IF(AND($C$7&lt;=Premissas!$D$65,$C$5&lt;=Premissas!$E$65),Premissas!$B$65,"Excede os planos (usar sob demanda)"))))</f>
         <v>Pro</v>
       </c>
-      <c r="D24" s="16" t="s">
-        <v>114</v>
+      <c r="D24" s="17" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
-      <c r="B25" s="17" t="s">
-        <v>115</v>
-      </c>
-      <c r="C25" s="29">
-        <f>IF(AND($C$7&lt;=Premissas!$D$50,$C$5&lt;=Premissas!$E$50),Premissas!$C$50,IF(AND($C$7&lt;=Premissas!$D$51,$C$5&lt;=Premissas!$E$51),Premissas!$C$51,IF(AND($C$7&lt;=Premissas!$D$52,$C$5&lt;=Premissas!$E$52),Premissas!$C$52,IF(AND($C$7&lt;=Premissas!$D$53,$C$5&lt;=Premissas!$E$53),Premissas!$C$53,$C$21))))</f>
+      <c r="B25" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25" s="30">
+        <f>IF(AND($C$7&lt;=Premissas!$D$62,$C$5&lt;=Premissas!$E$62),Premissas!$C$62,IF(AND($C$7&lt;=Premissas!$D$63,$C$5&lt;=Premissas!$E$63),Premissas!$C$63,IF(AND($C$7&lt;=Premissas!$D$64,$C$5&lt;=Premissas!$E$64),Premissas!$C$64,IF(AND($C$7&lt;=Premissas!$D$65,$C$5&lt;=Premissas!$E$65),Premissas!$C$65,$C$21))))</f>
         <v>15</v>
       </c>
       <c r="D25" s="4"/>
@@ -2717,74 +2921,74 @@
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="7" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
-      <c r="B28" s="17" t="s">
-        <v>117</v>
-      </c>
-      <c r="C28" s="29">
+      <c r="B28" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="C28" s="30">
         <f>C15-C21</f>
-        <v>102.63904014587496</v>
+        <v>275.44010087749984</v>
       </c>
       <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
-      <c r="B29" s="14" t="s">
-        <v>118</v>
-      </c>
-      <c r="C29" s="31">
+      <c r="B29" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C29" s="32">
         <f>IF(C21&gt;0,C15/C21,"n/a (CloudFront dentro do free tier)")</f>
-        <v>2.6422513781864359</v>
+        <v>1.1144177346084025</v>
       </c>
       <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
-      <c r="B30" s="14" t="s">
-        <v>119</v>
-      </c>
-      <c r="C30" s="28">
+      <c r="B30" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="C30" s="29">
         <f>C15-C25</f>
-        <v>150.13802264587497</v>
+        <v>2667.7601008775</v>
       </c>
       <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
-      <c r="B31" s="14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C31" s="32">
+      <c r="B31" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C31" s="33">
         <f>IF(C5&gt;0,C15/C5,0)</f>
-        <v>9.3945186216319976E-2</v>
+        <v>8.8049562285210256E-2</v>
       </c>
       <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
-      <c r="B32" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C32" s="32">
+      <c r="B32" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="C32" s="33">
         <f>IF(C5&gt;0,C21/C5,0)</f>
-        <v>3.5554976711111116E-2</v>
+        <v>7.9009476923076929E-2</v>
       </c>
       <c r="D32" s="4"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
-      <c r="B33" s="14" t="s">
-        <v>122</v>
-      </c>
-      <c r="C33" s="33">
+      <c r="B33" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="C33" s="34">
         <f>IF(C8&gt;0,C15/C8,0)</f>
-        <v>1.0900199514579206E-4</v>
+        <v>4.2583493664722223E-4</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -2796,23 +3000,23 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
-      <c r="B35" s="34" t="s">
-        <v>123</v>
-      </c>
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
+      <c r="B35" s="35" t="s">
+        <v>129</v>
+      </c>
+      <c r="C35" s="36"/>
+      <c r="D35" s="36"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="4"/>
-      <c r="B36" s="35"/>
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="36"/>
+      <c r="D36" s="36"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
-      <c r="B37" s="35"/>
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="36"/>
+      <c r="D37" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
docs(cost): use sa-east-1 prices, the production region
Production always runs in sa-east-1 for latency, so the cost workbook now
prices API Gateway requests, egress, S3 GET and Lambda there (AWS Price
List API) and defaults CloudFront users to South America.

With the initial estimate (~30 TB/month) API Gateway costs ~$4,380/month
against ~$3,140 on CloudFront pay-as-you-go (~1.4x): Sao Paulo egress is
$0.150/GB vs $0.110/GB on South America edges. ADR cost reading updated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/custo/apigw-vs-cloudfront.xlsx
+++ b/docs/custo/apigw-vs-cloudfront.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\apigw-transfer\.claude\worktrees\project-proposal-code-review-f9ab5f\docs\custo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0311FFE3-C7F4-44D2-AE7D-AFC432F1516C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4891E69F-16C7-4AFC-8439-F22653937378}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -149,7 +149,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>https://aws.amazon.com/lambda/pricing/ (arm64: 0,0000133334)</t>
+          <t>https://aws.amazon.com/lambda/pricing/ (sa-east-1, primeira faixa)</t>
         </r>
       </text>
     </comment>
@@ -163,7 +163,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>https://aws.amazon.com/s3/pricing/ (S3 Standard)</t>
+          <t>https://aws.amazon.com/s3/pricing/ (S3 Standard, sa-east-1, AWS Price List API)</t>
         </r>
       </text>
     </comment>
@@ -219,7 +219,7 @@
             <family val="2"/>
             <scheme val="minor"/>
           </rPr>
-          <t>CloudFront cobra pela região do edge que atende o usuário. API Gateway cobra pela região da API (us-east-1).</t>
+          <t>CloudFront cobra pela região do edge que atende o usuário. API Gateway cobra pela região da API (sa-east-1).</t>
         </r>
       </text>
     </comment>
@@ -280,7 +280,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="129">
   <si>
     <t>Consumo medido em produção</t>
   </si>
@@ -345,7 +345,7 @@
     <t>1. Aba Consumo: informe quantos dias o levantamento cobre (célula C2) e, por categoria de arquivo, downloads no período, tamanho médio, % com HEAD e % de requisições extras (retomadas/retries). Células amarelas com texto azul são entradas. As duas linhas preenchidas são uma estimativa inicial: substitua pelo levantamento.</t>
   </si>
   <si>
-    <t>2. Aba Premissas: escolha a região dos usuários (América do Norte ou América do Sul), que define o preço do CloudFront. O API Gateway usa o preço de us-east-1. Demais preços e parâmetros são editáveis (texto azul).</t>
+    <t>2. Aba Premissas: escolha a região dos usuários (América do Norte ou América do Sul), que define o preço do CloudFront. O API Gateway usa o preço de sa-east-1 (região de produção). Demais preços e parâmetros são editáveis (texto azul).</t>
   </si>
   <si>
     <t>3. Aba Comparativo: resultado mensal, sem nada a preencher.</t>
@@ -393,7 +393,7 @@
     <t>Lambda: https://aws.amazon.com/lambda/pricing/</t>
   </si>
   <si>
-    <t>Preços de referência (API Gateway/S3/Lambda em us-east-1; CloudFront por região), conferidos em 2026-09-13. Confirmar antes de decidir.</t>
+    <t>Preços de referência (API Gateway/S3/Lambda em sa-east-1, região de produção; CloudFront por região), conferidos em 2026-09-13. Confirmar antes de decidir.</t>
   </si>
   <si>
     <t>Premissas e preços</t>
@@ -450,7 +450,7 @@
     <t>Região dos usuários (define a tabela de preço do CloudFront)</t>
   </si>
   <si>
-    <t>América do Norte</t>
+    <t>América do Sul</t>
   </si>
   <si>
     <t>Preço por 10.000 requisições HTTPS ($) - América do Norte</t>
@@ -474,10 +474,7 @@
     <t>Preço ($)</t>
   </si>
   <si>
-    <t>Primeiros 333 milhões</t>
-  </si>
-  <si>
-    <t>Próximos 667 milhões</t>
+    <t>Primeiro 1 bilhão</t>
   </si>
   <si>
     <t>Próximos 19 bilhões</t>
@@ -486,7 +483,7 @@
     <t>Acima de 20 bilhões</t>
   </si>
   <si>
-    <t>Fonte: https://aws.amazon.com/api-gateway/pricing/. Última faixa com 'Até' = 1E+12 (sem limite).</t>
+    <t>Fonte: https://aws.amazon.com/api-gateway/pricing/ (sa-east-1, AWS Price List API). Última faixa com 'Até' = 1E+12 (sem limite).</t>
   </si>
   <si>
     <t>API Gateway: transferência para a internet por mês (preço por GB)</t>
@@ -510,7 +507,7 @@
     <t>Acima de 150 TB</t>
   </si>
   <si>
-    <t>Fonte: https://aws.amazon.com/api-gateway/pricing/ (mesma tabela de transferência do EC2, us-east-1). Última faixa com 'Até' = 1E+12 (sem limite).</t>
+    <t>Fonte: https://aws.amazon.com/api-gateway/pricing/ (transferência para a internet a partir de sa-east-1, AWS Price List API). Última faixa com 'Até' = 1E+12 (sem limite).</t>
   </si>
   <si>
     <t>CloudFront sob demanda - América do Norte: transferência por mês (preço por GB, após free tier)</t>
@@ -1182,7 +1179,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="2:2" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" ht="42.75" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
@@ -1286,7 +1283,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
@@ -1440,7 +1437,7 @@
         <v>50</v>
       </c>
       <c r="C15" s="12">
-        <v>4.0000000000000002E-4</v>
+        <v>5.5999999999999995E-4</v>
       </c>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
@@ -1560,10 +1557,10 @@
         <v>0</v>
       </c>
       <c r="D26" s="9">
-        <v>333</v>
+        <v>1000</v>
       </c>
       <c r="E26" s="12">
-        <v>3.5</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1572,13 +1569,13 @@
         <v>65</v>
       </c>
       <c r="C27" s="9">
-        <v>333</v>
+        <v>1000</v>
       </c>
       <c r="D27" s="9">
-        <v>1000</v>
+        <v>20000</v>
       </c>
       <c r="E27" s="12">
-        <v>2.8</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1587,68 +1584,68 @@
         <v>66</v>
       </c>
       <c r="C28" s="9">
-        <v>1000</v>
+        <v>20000</v>
       </c>
       <c r="D28" s="9">
-        <v>20000</v>
+        <v>1000000000000</v>
       </c>
       <c r="E28" s="12">
-        <v>2.38</v>
+        <v>2.29</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="9">
-        <v>20000</v>
-      </c>
-      <c r="D29" s="9">
-        <v>1000000000000</v>
-      </c>
-      <c r="E29" s="12">
-        <v>1.51</v>
-      </c>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
-      <c r="B30" s="6" t="s">
-        <v>68</v>
-      </c>
+      <c r="B30" s="4"/>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
+      <c r="B31" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C32" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
+      <c r="D32" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
-      <c r="B33" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D33" s="14" t="s">
+      <c r="B33" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="E33" s="14" t="s">
-        <v>63</v>
+      <c r="C33" s="9">
+        <v>0</v>
+      </c>
+      <c r="D33" s="9">
+        <v>10240</v>
+      </c>
+      <c r="E33" s="12">
+        <v>0.15</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
@@ -1657,13 +1654,13 @@
         <v>72</v>
       </c>
       <c r="C34" s="9">
-        <v>0</v>
+        <v>10240</v>
       </c>
       <c r="D34" s="9">
-        <v>10240</v>
+        <v>51200</v>
       </c>
       <c r="E34" s="12">
-        <v>0.09</v>
+        <v>0.13800000000000001</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1672,13 +1669,13 @@
         <v>73</v>
       </c>
       <c r="C35" s="9">
-        <v>10240</v>
+        <v>51200</v>
       </c>
       <c r="D35" s="9">
-        <v>51200</v>
+        <v>153600</v>
       </c>
       <c r="E35" s="12">
-        <v>8.5000000000000006E-2</v>
+        <v>0.126</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1687,68 +1684,68 @@
         <v>74</v>
       </c>
       <c r="C36" s="9">
-        <v>51200</v>
+        <v>153600</v>
       </c>
       <c r="D36" s="9">
-        <v>153600</v>
+        <v>1000000000000</v>
       </c>
       <c r="E36" s="12">
-        <v>7.0000000000000007E-2</v>
+        <v>0.114</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C37" s="9">
-        <v>153600</v>
-      </c>
-      <c r="D37" s="9">
-        <v>1000000000000</v>
-      </c>
-      <c r="E37" s="12">
-        <v>0.05</v>
-      </c>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
-      <c r="B38" s="6" t="s">
-        <v>76</v>
-      </c>
+      <c r="B38" s="4"/>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4"/>
-      <c r="D39" s="4"/>
-      <c r="E39" s="4"/>
+      <c r="B39" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
-      <c r="B40" s="7" t="s">
-        <v>77</v>
-      </c>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
+      <c r="B40" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D40" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E40" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
-      <c r="B41" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D41" s="14" t="s">
+      <c r="B41" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="E41" s="14" t="s">
-        <v>63</v>
+      <c r="C41" s="9">
+        <v>0</v>
+      </c>
+      <c r="D41" s="9">
+        <v>10240</v>
+      </c>
+      <c r="E41" s="12">
+        <v>8.5000000000000006E-2</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1757,13 +1754,13 @@
         <v>72</v>
       </c>
       <c r="C42" s="9">
-        <v>0</v>
+        <v>10240</v>
       </c>
       <c r="D42" s="9">
-        <v>10240</v>
+        <v>51200</v>
       </c>
       <c r="E42" s="12">
-        <v>8.5000000000000006E-2</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1772,28 +1769,28 @@
         <v>73</v>
       </c>
       <c r="C43" s="9">
-        <v>10240</v>
+        <v>51200</v>
       </c>
       <c r="D43" s="9">
-        <v>51200</v>
+        <v>153600</v>
       </c>
       <c r="E43" s="12">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C44" s="9">
-        <v>51200</v>
+        <v>153600</v>
       </c>
       <c r="D44" s="9">
-        <v>153600</v>
+        <v>512000</v>
       </c>
       <c r="E44" s="12">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1802,13 +1799,13 @@
         <v>78</v>
       </c>
       <c r="C45" s="9">
-        <v>153600</v>
+        <v>512000</v>
       </c>
       <c r="D45" s="9">
-        <v>512000</v>
+        <v>1048576</v>
       </c>
       <c r="E45" s="12">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1817,68 +1814,68 @@
         <v>79</v>
       </c>
       <c r="C46" s="9">
-        <v>512000</v>
+        <v>1048576</v>
       </c>
       <c r="D46" s="9">
-        <v>1048576</v>
+        <v>1000000000000</v>
       </c>
       <c r="E46" s="12">
-        <v>0.03</v>
+        <v>2.5000000000000001E-2</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="4"/>
-      <c r="B47" s="15" t="s">
+      <c r="B47" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C47" s="9">
-        <v>1048576</v>
-      </c>
-      <c r="D47" s="9">
-        <v>1000000000000</v>
-      </c>
-      <c r="E47" s="12">
-        <v>2.5000000000000001E-2</v>
-      </c>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="4"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
-      <c r="B48" s="6" t="s">
-        <v>81</v>
-      </c>
+      <c r="B48" s="4"/>
       <c r="C48" s="4"/>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
-      <c r="C49" s="4"/>
-      <c r="D49" s="4"/>
-      <c r="E49" s="4"/>
+      <c r="B49" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
-      <c r="B50" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
+      <c r="B50" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D50" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E50" s="14" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
-      <c r="B51" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C51" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="D51" s="14" t="s">
+      <c r="B51" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="E51" s="14" t="s">
-        <v>63</v>
+      <c r="C51" s="9">
+        <v>0</v>
+      </c>
+      <c r="D51" s="9">
+        <v>10240</v>
+      </c>
+      <c r="E51" s="12">
+        <v>0.11</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -1887,13 +1884,13 @@
         <v>72</v>
       </c>
       <c r="C52" s="9">
-        <v>0</v>
+        <v>10240</v>
       </c>
       <c r="D52" s="9">
-        <v>10240</v>
+        <v>51200</v>
       </c>
       <c r="E52" s="12">
-        <v>0.11</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -1902,28 +1899,28 @@
         <v>73</v>
       </c>
       <c r="C53" s="9">
-        <v>10240</v>
+        <v>51200</v>
       </c>
       <c r="D53" s="9">
-        <v>51200</v>
+        <v>153600</v>
       </c>
       <c r="E53" s="12">
-        <v>0.105</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="4"/>
       <c r="B54" s="15" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C54" s="9">
-        <v>51200</v>
+        <v>153600</v>
       </c>
       <c r="D54" s="9">
-        <v>153600</v>
+        <v>512000</v>
       </c>
       <c r="E54" s="12">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -1932,13 +1929,13 @@
         <v>78</v>
       </c>
       <c r="C55" s="9">
-        <v>153600</v>
+        <v>512000</v>
       </c>
       <c r="D55" s="9">
-        <v>512000</v>
+        <v>1048576</v>
       </c>
       <c r="E55" s="12">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -1947,68 +1944,68 @@
         <v>79</v>
       </c>
       <c r="C56" s="9">
-        <v>512000</v>
+        <v>1048576</v>
       </c>
       <c r="D56" s="9">
-        <v>1048576</v>
+        <v>1000000000000</v>
       </c>
       <c r="E56" s="12">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="4"/>
-      <c r="B57" s="15" t="s">
-        <v>80</v>
-      </c>
-      <c r="C57" s="9">
-        <v>1048576</v>
-      </c>
-      <c r="D57" s="9">
-        <v>1000000000000</v>
-      </c>
-      <c r="E57" s="12">
-        <v>0.05</v>
-      </c>
+      <c r="B57" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57" s="4"/>
+      <c r="D57" s="4"/>
+      <c r="E57" s="4"/>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="4"/>
-      <c r="B58" s="6" t="s">
-        <v>83</v>
-      </c>
+      <c r="B58" s="4"/>
       <c r="C58" s="4"/>
       <c r="D58" s="4"/>
       <c r="E58" s="4"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
-      <c r="B59" s="4"/>
-      <c r="C59" s="4"/>
-      <c r="D59" s="4"/>
-      <c r="E59" s="4"/>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B59" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C59" s="8"/>
+      <c r="D59" s="8"/>
+      <c r="E59" s="8"/>
+    </row>
+    <row r="60" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="4"/>
-      <c r="B60" s="7" t="s">
+      <c r="B60" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="C60" s="8"/>
-      <c r="D60" s="8"/>
-      <c r="E60" s="8"/>
-    </row>
-    <row r="61" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="C60" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="D60" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="E60" s="14" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
-      <c r="B61" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C61" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D61" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="E61" s="14" t="s">
+      <c r="B61" s="16" t="s">
         <v>88</v>
+      </c>
+      <c r="C61" s="11">
+        <v>0</v>
+      </c>
+      <c r="D61" s="9">
+        <v>1000000</v>
+      </c>
+      <c r="E61" s="9">
+        <v>100</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -2017,13 +2014,13 @@
         <v>89</v>
       </c>
       <c r="C62" s="11">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D62" s="9">
-        <v>1000000</v>
+        <v>10000000</v>
       </c>
       <c r="E62" s="9">
-        <v>100</v>
+        <v>51200</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
@@ -2032,10 +2029,10 @@
         <v>90</v>
       </c>
       <c r="C63" s="11">
-        <v>15</v>
+        <v>200</v>
       </c>
       <c r="D63" s="9">
-        <v>10000000</v>
+        <v>125000000</v>
       </c>
       <c r="E63" s="9">
         <v>51200</v>
@@ -2047,38 +2044,23 @@
         <v>91</v>
       </c>
       <c r="C64" s="11">
-        <v>200</v>
+        <v>1000</v>
       </c>
       <c r="D64" s="9">
-        <v>125000000</v>
+        <v>500000000</v>
       </c>
       <c r="E64" s="9">
         <v>51200</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="C65" s="11">
-        <v>1000</v>
-      </c>
-      <c r="D65" s="9">
-        <v>500000000</v>
-      </c>
-      <c r="E65" s="9">
-        <v>51200</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" ht="42.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="4"/>
-      <c r="B66" s="17" t="s">
-        <v>93</v>
-      </c>
-      <c r="C66" s="4"/>
-      <c r="D66" s="4"/>
-      <c r="E66" s="4"/>
+      <c r="C65" s="4"/>
+      <c r="D65" s="4"/>
+      <c r="E65" s="4"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -2664,7 +2646,7 @@
     <row r="1" spans="1:4" ht="18" x14ac:dyDescent="0.25">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C1" s="4"/>
       <c r="D1" s="4"/>
@@ -2672,7 +2654,7 @@
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="4"/>
       <c r="B2" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
@@ -2686,7 +2668,7 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -2694,20 +2676,20 @@
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4"/>
       <c r="B5" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C5" s="27">
         <f>Consumo!$G$20*(Premissas!$C$5/Consumo!$C$2)</f>
         <v>30468.75</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
       <c r="B6" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" s="28">
         <f>Consumo!$I$20*(Premissas!$C$5/Consumo!$C$2)</f>
@@ -2718,7 +2700,7 @@
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4"/>
       <c r="B7" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" s="28">
         <f>Consumo!$J$20*(Premissas!$C$5/Consumo!$C$2)</f>
@@ -2729,7 +2711,7 @@
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
       <c r="B8" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="28">
         <f>Consumo!$C$20*(Premissas!$C$5/Consumo!$C$2)</f>
@@ -2746,7 +2728,7 @@
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="4"/>
       <c r="B10" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -2754,61 +2736,61 @@
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="4"/>
       <c r="B11" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="C11" s="29">
+        <f>SUMPRODUCT((($C$6/1000000)&gt;Premissas!$C$26:$C$28)*((($C$6/1000000)-Premissas!$C$26:$C$28)-(($C$6/1000000)&gt;Premissas!$D$26:$D$28)*(($C$6/1000000)-Premissas!$D$26:$D$28))*Premissas!$E$26:$E$28)</f>
+        <v>44.752499999999998</v>
+      </c>
+      <c r="D11" s="17" t="s">
         <v>103</v>
-      </c>
-      <c r="C11" s="29">
-        <f>SUMPRODUCT((($C$6/1000000)&gt;Premissas!$C$26:$C$29)*((($C$6/1000000)-Premissas!$C$26:$C$29)-(($C$6/1000000)&gt;Premissas!$D$26:$D$29)*(($C$6/1000000)-Premissas!$D$26:$D$29))*Premissas!$E$26:$E$29)</f>
-        <v>36.854999999999997</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="4"/>
       <c r="B12" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="C12" s="29">
+        <f>SUMPRODUCT(($C$5&gt;Premissas!$C$33:$C$36)*(($C$5-Premissas!$C$33:$C$36)-($C$5&gt;Premissas!$D$33:$D$36)*($C$5-Premissas!$D$33:$D$36))*Premissas!$E$33:$E$36)</f>
+        <v>4327.5675000000001</v>
+      </c>
+      <c r="D12" s="17" t="s">
         <v>105</v>
-      </c>
-      <c r="C12" s="29">
-        <f>SUMPRODUCT(($C$5&gt;Premissas!$C$34:$C$37)*(($C$5-Premissas!$C$34:$C$37)-($C$5&gt;Premissas!$D$34:$D$37)*($C$5-Premissas!$D$34:$D$37))*Premissas!$E$34:$E$37)</f>
-        <v>2641.0437499999998</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
       <c r="B13" s="15" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" s="29">
         <f>$C$6/1000*Premissas!$C$15</f>
-        <v>4.2120000000000006</v>
+        <v>5.8967999999999998</v>
       </c>
       <c r="D13" s="4"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="4"/>
       <c r="B14" s="15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C14" s="29">
         <f>$C$6*(1-Premissas!$C$9)*(Premissas!$C$12/1000000+(Premissas!$C$10/1024)*(Premissas!$C$11/1000)*Premissas!$C$13)</f>
         <v>0.64935087749999987</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="4"/>
       <c r="B15" s="18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C15" s="30">
         <f>SUM(C11:C14)</f>
-        <v>2682.7601008775</v>
+        <v>4378.8661508775003</v>
       </c>
       <c r="D15" s="4"/>
     </row>
@@ -2821,7 +2803,7 @@
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="4"/>
       <c r="B17" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C17" s="8"/>
       <c r="D17" s="8"/>
@@ -2829,48 +2811,48 @@
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="4"/>
       <c r="B18" s="15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C18" s="29">
         <f>MAX(0,$C$7-Premissas!$C$19)/10000*IF((Premissas!$C$20="América do Sul"),Premissas!$C$22,Premissas!$C$21)</f>
         <v>0</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="4"/>
       <c r="B19" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="29">
+        <f>IF((Premissas!$C$20="América do Sul"),SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$51:$C$56)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$51:$C$56)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$51:$D$56)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$51:$D$56))*Premissas!$E$51:$E$56),SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$41:$C$46)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$41:$C$46)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$41:$D$46)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$41:$D$46))*Premissas!$E$41:$E$46))</f>
+        <v>3142.8987500000003</v>
+      </c>
+      <c r="D19" s="17" t="s">
         <v>114</v>
-      </c>
-      <c r="C19" s="29">
-        <f>IF((Premissas!$C$20="América do Sul"),SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$52:$C$57)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$52:$C$57)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$52:$D$57)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$52:$D$57))*Premissas!$E$52:$E$57),SUMPRODUCT((MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$C$42:$C$47)*((MAX(0,$C$5-Premissas!$C$18)-Premissas!$C$42:$C$47)-(MAX(0,$C$5-Premissas!$C$18)&gt;Premissas!$D$42:$D$47)*(MAX(0,$C$5-Premissas!$C$18)-Premissas!$D$42:$D$47))*Premissas!$E$42:$E$47))</f>
-        <v>2406.7800000000002</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="4"/>
       <c r="B20" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C20" s="29">
         <f>$C$7*(1-Premissas!$C$17)/1000*Premissas!$C$15</f>
-        <v>0.53999999999999992</v>
+        <v>0.75599999999999978</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="4"/>
       <c r="B21" s="18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C21" s="30">
         <f>SUM(C18:C20)</f>
-        <v>2407.3200000000002</v>
+        <v>3143.6547500000001</v>
       </c>
       <c r="D21" s="4"/>
     </row>
@@ -2883,7 +2865,7 @@
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="4"/>
       <c r="B23" s="7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8"/>
@@ -2891,23 +2873,23 @@
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="4"/>
       <c r="B24" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="C24" s="31" t="str">
+        <f>IF(AND($C$7&lt;=Premissas!$D$61,$C$5&lt;=Premissas!$E$61),Premissas!$B$61,IF(AND($C$7&lt;=Premissas!$D$62,$C$5&lt;=Premissas!$E$62),Premissas!$B$62,IF(AND($C$7&lt;=Premissas!$D$63,$C$5&lt;=Premissas!$E$63),Premissas!$B$63,IF(AND($C$7&lt;=Premissas!$D$64,$C$5&lt;=Premissas!$E$64),Premissas!$B$64,"Excede os planos (usar sob demanda)"))))</f>
+        <v>Pro</v>
+      </c>
+      <c r="D24" s="17" t="s">
         <v>119</v>
-      </c>
-      <c r="C24" s="31" t="str">
-        <f>IF(AND($C$7&lt;=Premissas!$D$62,$C$5&lt;=Premissas!$E$62),Premissas!$B$62,IF(AND($C$7&lt;=Premissas!$D$63,$C$5&lt;=Premissas!$E$63),Premissas!$B$63,IF(AND($C$7&lt;=Premissas!$D$64,$C$5&lt;=Premissas!$E$64),Premissas!$B$64,IF(AND($C$7&lt;=Premissas!$D$65,$C$5&lt;=Premissas!$E$65),Premissas!$B$65,"Excede os planos (usar sob demanda)"))))</f>
-        <v>Pro</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="4"/>
       <c r="B25" s="18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C25" s="30">
-        <f>IF(AND($C$7&lt;=Premissas!$D$62,$C$5&lt;=Premissas!$E$62),Premissas!$C$62,IF(AND($C$7&lt;=Premissas!$D$63,$C$5&lt;=Premissas!$E$63),Premissas!$C$63,IF(AND($C$7&lt;=Premissas!$D$64,$C$5&lt;=Premissas!$E$64),Premissas!$C$64,IF(AND($C$7&lt;=Premissas!$D$65,$C$5&lt;=Premissas!$E$65),Premissas!$C$65,$C$21))))</f>
+        <f>IF(AND($C$7&lt;=Premissas!$D$61,$C$5&lt;=Premissas!$E$61),Premissas!$C$61,IF(AND($C$7&lt;=Premissas!$D$62,$C$5&lt;=Premissas!$E$62),Premissas!$C$62,IF(AND($C$7&lt;=Premissas!$D$63,$C$5&lt;=Premissas!$E$63),Premissas!$C$63,IF(AND($C$7&lt;=Premissas!$D$64,$C$5&lt;=Premissas!$E$64),Premissas!$C$64,$C$21))))</f>
         <v>15</v>
       </c>
       <c r="D25" s="4"/>
@@ -2921,7 +2903,7 @@
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="4"/>
       <c r="B27" s="7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C27" s="8"/>
       <c r="D27" s="8"/>
@@ -2929,66 +2911,66 @@
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="4"/>
       <c r="B28" s="18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C28" s="30">
         <f>C15-C21</f>
-        <v>275.44010087749984</v>
+        <v>1235.2114008775002</v>
       </c>
       <c r="D28" s="4"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="4"/>
       <c r="B29" s="15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C29" s="32">
         <f>IF(C21&gt;0,C15/C21,"n/a (CloudFront dentro do free tier)")</f>
-        <v>1.1144177346084025</v>
+        <v>1.3929220919941989</v>
       </c>
       <c r="D29" s="4"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="4"/>
       <c r="B30" s="15" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C30" s="29">
         <f>C15-C25</f>
-        <v>2667.7601008775</v>
+        <v>4363.8661508775003</v>
       </c>
       <c r="D30" s="4"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="4"/>
       <c r="B31" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C31" s="33">
         <f>IF(C5&gt;0,C15/C5,0)</f>
-        <v>8.8049562285210256E-2</v>
+        <v>0.14371663264418463</v>
       </c>
       <c r="D31" s="4"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="4"/>
       <c r="B32" s="15" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C32" s="33">
         <f>IF(C5&gt;0,C21/C5,0)</f>
-        <v>7.9009476923076929E-2</v>
+        <v>0.10317636102564103</v>
       </c>
       <c r="D32" s="4"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="4"/>
       <c r="B33" s="15" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C33" s="34">
         <f>IF(C8&gt;0,C15/C8,0)</f>
-        <v>4.2583493664722223E-4</v>
+        <v>6.9505811918690484E-4</v>
       </c>
       <c r="D33" s="4"/>
     </row>
@@ -3001,7 +2983,7 @@
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="35" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C35" s="36"/>
       <c r="D35" s="36"/>

</xml_diff>